<commit_message>
Added new RDF data schemes and visual schemes, fixed XLSX spreadsheets for economy-table65-67
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table66.xlsx
+++ b/sources/table_normalization/xlsx/economy-table66.xlsx
@@ -457,11 +457,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="5">
-    <numFmt numFmtId="167" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="[$-1009]d\-mmm\-yy;@"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0"/>
-    <numFmt numFmtId="170" formatCode="0.0%"/>
-    <numFmt numFmtId="171" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="[$-1009]d\-mmm\-yy;@"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -587,7 +587,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -609,6 +609,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -792,7 +798,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -812,7 +818,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -821,7 +827,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -831,48 +837,48 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="15" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="9" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -886,7 +892,7 @@
     <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -911,19 +917,19 @@
     <xf numFmtId="10" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="16" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="16" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="9" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="9" fillId="4" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2539,11 +2545,11 @@
         <v>17</v>
       </c>
       <c r="H36" s="23">
-        <f t="shared" ref="H36:H67" si="4">G36/$G$2</f>
+        <f t="shared" ref="H36:H60" si="4">G36/$G$2</f>
         <v>6.8728522336769802E-3</v>
       </c>
       <c r="I36" s="29">
-        <f t="shared" ref="I36:I67" si="5">$I$1*H36</f>
+        <f t="shared" ref="I36:I60" si="5">$I$1*H36</f>
         <v>11.821305841924399</v>
       </c>
     </row>

</xml_diff>